<commit_message>
trabajos de prueba para montar version candidate en ritrama!
</commit_message>
<xml_diff>
--- a/bin/Debug/net9.0-windows/detalle_paleta.xlsx
+++ b/bin/Debug/net9.0-windows/detalle_paleta.xlsx
@@ -34,18 +34,16 @@
     <x:t>Kilo_Bruto</x:t>
   </x:si>
   <x:si>
-    <x:t>45</x:t>
-  </x:si>
-  <x:si>
-    <x:t>69</x:t>
-  </x:si>
-  <x:si>
-    <x:t>50X50</x:t>
-  </x:si>
-  <x:si>
-    <x:t>DFNSA.FSFSDFJÑKÑ.KSAJFH
-SF-SHFKJSHFÑKSADJFSÑKJFH
-SDLFKHSLFKSÑAFHASDÑF</x:t>
+    <x:t>2</x:t>
+  </x:si>
+  <x:si>
+    <x:t>1050</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">50X50     </x:t>
+  </x:si>
+  <x:si>
+    <x:t>DETAILS PALETA</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -107,17 +105,13 @@
       <x:protection locked="1" hidden="0"/>
     </x:xf>
   </x:cellStyleXfs>
-  <x:cellXfs count="3">
+  <x:cellXfs count="2">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
       <x:alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <x:protection locked="1" hidden="0"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
       <x:alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <x:protection locked="1" hidden="0"/>
     </x:xf>
   </x:cellXfs>
@@ -420,8 +414,8 @@
   <x:cols>
     <x:col min="1" max="1" width="8.282054" style="0" customWidth="1"/>
     <x:col min="2" max="2" width="13.853482" style="0" customWidth="1"/>
-    <x:col min="3" max="3" width="7.853482" style="0" customWidth="1"/>
-    <x:col min="4" max="4" width="26.139196" style="0" customWidth="1"/>
+    <x:col min="3" max="3" width="8.567768" style="0" customWidth="1"/>
+    <x:col min="4" max="4" width="15.139196" style="0" customWidth="1"/>
     <x:col min="5" max="5" width="9.567768" style="0" customWidth="1"/>
     <x:col min="6" max="6" width="10.282054" style="0" customWidth="1"/>
   </x:cols>
@@ -456,14 +450,14 @@
       <x:c r="C2" s="0" t="s">
         <x:v>8</x:v>
       </x:c>
-      <x:c r="D2" s="2" t="s">
+      <x:c r="D2" s="0" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="E2" s="0">
-        <x:v>850</x:v>
+        <x:v>1000</x:v>
       </x:c>
       <x:c r="F2" s="0">
-        <x:v>1250</x:v>
+        <x:v>1200</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>